<commit_message>
05/08/2026 19:39 note update
</commit_message>
<xml_diff>
--- a/Documentation Data/LCAS Vicon Temperature Tracker.xlsx
+++ b/Documentation Data/LCAS Vicon Temperature Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newwb\Documents\brain\professional\university\LCAS\EPSURIS Internship (Vicon)\Public Files\Documentation Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F595C417-1755-420E-8DE6-9B7FFA50463C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9030D01B-764E-4BC0-A0CE-D8E29AA06B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="4" r:id="rId1"/>
@@ -69,60 +69,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{C01FFB04-8F84-491C-BB2E-65383C0F8D44}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Daniel Newby:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-persistently slow to auto-stop when calibrating</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O3" authorId="0" shapeId="0" xr:uid="{17C8BC38-A956-4D7F-998B-6CD76E9EE7EB}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Daniel Newby:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-persistently slow to auto-stop when calibrating</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -144,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="52">
   <si>
     <t>Starting Time</t>
   </si>
@@ -469,6 +421,21 @@
     <t>Recording with camera temperature tracking script from this day</t>
   </si>
   <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Camera by ID</t>
+  </si>
+  <si>
+    <t>This is a dev troubleshooting record for the camera temperature script, checking which cameras are dropped from readings</t>
+  </si>
+  <si>
+    <t>Cameras Missing from Temperature Script Log</t>
+  </si>
+  <si>
+    <t>(04/08 is first day recording these errors)</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">(tested script against non-active system configs) - on selecting VCS on init, 1 cam active, temp not shown. </t>
     </r>
@@ -535,23 +502,24 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>)</t>
+      <t xml:space="preserve">)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>time to ready wasn't faster than yesterday despite higher starting temp</t>
     </r>
   </si>
   <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Camera by ID</t>
-  </si>
-  <si>
-    <t>This is a dev troubleshooting record for the camera temperature script, checking which cameras are dropped from readings</t>
-  </si>
-  <si>
-    <t>Cameras Missing from Temperature Script Log</t>
-  </si>
-  <si>
-    <t>(04/08 is first day recording these errors)</t>
+    <t>startup time may be off by 30 seconds, recorded after start</t>
   </si>
 </sst>
 </file>
@@ -826,7 +794,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor rgb="FFBDD7EE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -962,7 +930,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1028,9 +996,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1058,9 +1023,6 @@
     <xf numFmtId="0" fontId="22" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1076,6 +1038,19 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1084,17 +1059,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1127,6 +1091,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFBDD7EE"/>
       <color rgb="FF1F4E78"/>
       <color rgb="FFC65911"/>
     </mruColors>
@@ -1292,6 +1257,9 @@
                 <c:pt idx="9">
                   <c:v>46238</c:v>
                 </c:pt>
+                <c:pt idx="10">
+                  <c:v>46239</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1329,6 +1297,9 @@
                   <c:v>23.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>24.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>24.5</c:v>
                 </c:pt>
               </c:numCache>
@@ -1413,6 +1384,9 @@
                 <c:pt idx="9">
                   <c:v>46238</c:v>
                 </c:pt>
+                <c:pt idx="10">
+                  <c:v>46239</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1450,10 +1424,10 @@
                   <c:v>21.216666666666654</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>21.066666666666627</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>19.600000000000026</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -3201,7 +3175,7 @@
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Instructions"/>
-      <sheetName val="Lists"/>
+      <sheetName val="Data-Lists"/>
       <sheetName val="Camera Labelling"/>
       <sheetName val="Log"/>
       <sheetName val="Daily Summary"/>
@@ -3697,16 +3671,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
       <c r="I1" s="19" t="s">
         <v>18</v>
       </c>
@@ -5622,370 +5596,682 @@
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
+        <v>46238</v>
+      </c>
       <c r="C75" s="9">
         <f>_xlfn.XLOOKUP(Log!A75, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E75" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D75" s="9">
+        <v>0.43334490740740739</v>
+      </c>
+      <c r="E75" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H75" s="2" t="str">
+        <v>5.0166666666665982</v>
+      </c>
+      <c r="F75" s="7">
+        <v>38</v>
+      </c>
+      <c r="G75" s="2">
+        <v>39</v>
+      </c>
+      <c r="H75" s="2">
         <f t="shared" si="3"/>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
+        <v>46238</v>
+      </c>
       <c r="C76" s="9">
         <f>_xlfn.XLOOKUP(Log!A76, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E76" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D76" s="9">
+        <v>0.43752314814814813</v>
+      </c>
+      <c r="E76" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H76" s="2" t="str">
+        <v>11.033333333333273</v>
+      </c>
+      <c r="F76" s="7">
+        <v>44</v>
+      </c>
+      <c r="G76" s="2">
+        <v>45</v>
+      </c>
+      <c r="H76" s="2">
         <f t="shared" si="3"/>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
+        <v>46238</v>
+      </c>
       <c r="C77" s="9">
         <f>_xlfn.XLOOKUP(Log!A77, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E77" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D77" s="9">
+        <v>0.43892361111111111</v>
+      </c>
+      <c r="E77" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H77" s="2" t="str">
+        <v>13.049999999999962</v>
+      </c>
+      <c r="F77" s="7">
+        <v>47</v>
+      </c>
+      <c r="G77" s="2">
+        <v>48</v>
+      </c>
+      <c r="H77" s="2">
         <f t="shared" si="3"/>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
+        <v>46238</v>
+      </c>
       <c r="C78" s="9">
         <f>_xlfn.XLOOKUP(Log!A78, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E78" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D78" s="9">
+        <v>0.4403125</v>
+      </c>
+      <c r="E78" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H78" s="2" t="str">
+        <v>15.049999999999955</v>
+      </c>
+      <c r="F78" s="7">
+        <v>47</v>
+      </c>
+      <c r="G78" s="2">
+        <v>49</v>
+      </c>
+      <c r="H78" s="2">
         <f t="shared" si="3"/>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
+        <v>46238</v>
+      </c>
       <c r="C79" s="9">
         <f>_xlfn.XLOOKUP(Log!A79, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E79" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D79" s="9">
+        <v>0.44310185185185186</v>
+      </c>
+      <c r="E79" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H79" s="2" t="str">
+        <v>19.066666666666634</v>
+      </c>
+      <c r="F79" s="7">
+        <v>49</v>
+      </c>
+      <c r="G79" s="2">
+        <v>52</v>
+      </c>
+      <c r="H79" s="2">
         <f t="shared" si="3"/>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
+        <v>46238</v>
+      </c>
       <c r="C80" s="9">
         <f>_xlfn.XLOOKUP(Log!A80, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E80" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D80" s="9">
+        <v>0.44449074074074074</v>
+      </c>
+      <c r="E80" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H80" s="2" t="str">
+        <v>21.066666666666627</v>
+      </c>
+      <c r="F80" s="7">
+        <v>51</v>
+      </c>
+      <c r="G80" s="2">
+        <v>52</v>
+      </c>
+      <c r="H80" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
+        <v>46238</v>
+      </c>
       <c r="C81" s="9">
         <f>_xlfn.XLOOKUP(Log!A81, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E81" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D81" s="9">
+        <v>0.44589120370370372</v>
+      </c>
+      <c r="E81" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H81" s="2" t="str">
+        <v>23.083333333333318</v>
+      </c>
+      <c r="F81" s="7">
+        <v>52</v>
+      </c>
+      <c r="G81" s="2">
+        <v>55</v>
+      </c>
+      <c r="H81" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A82" s="1">
+        <v>46238</v>
+      </c>
       <c r="C82" s="9">
         <f>_xlfn.XLOOKUP(Log!A82, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E82" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D82" s="9">
+        <v>0.4472800925925926</v>
+      </c>
+      <c r="E82" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H82" s="2" t="str">
+        <v>25.083333333333311</v>
+      </c>
+      <c r="F82" s="7">
+        <v>52</v>
+      </c>
+      <c r="G82" s="2">
+        <v>55</v>
+      </c>
+      <c r="H82" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A83" s="1">
+        <v>46238</v>
+      </c>
       <c r="C83" s="9">
         <f>_xlfn.XLOOKUP(Log!A83, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E83" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D83" s="9">
+        <v>0.44866898148148149</v>
+      </c>
+      <c r="E83" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H83" s="2" t="str">
+        <v>27.083333333333304</v>
+      </c>
+      <c r="F83" s="7">
+        <v>54</v>
+      </c>
+      <c r="G83" s="2">
+        <v>55</v>
+      </c>
+      <c r="H83" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A84" s="1">
+        <v>46238</v>
+      </c>
       <c r="C84" s="9">
         <f>_xlfn.XLOOKUP(Log!A84, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E84" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D84" s="9">
+        <v>0.45005787037037037</v>
+      </c>
+      <c r="E84" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H84" s="2" t="str">
+        <v>29.083333333333297</v>
+      </c>
+      <c r="F84" s="7">
+        <v>54</v>
+      </c>
+      <c r="G84" s="2">
+        <v>55</v>
+      </c>
+      <c r="H84" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="85" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
+        <v>46238</v>
+      </c>
       <c r="C85" s="9">
         <f>_xlfn.XLOOKUP(Log!A85, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E85" s="6" t="str">
+        <v>0.42986111111111114</v>
+      </c>
+      <c r="D85" s="9">
+        <v>0.45145833333333335</v>
+      </c>
+      <c r="E85" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H85" s="2" t="str">
+        <v>31.099999999999987</v>
+      </c>
+      <c r="F85" s="7">
+        <v>55</v>
+      </c>
+      <c r="G85" s="2">
+        <v>58</v>
+      </c>
+      <c r="H85" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="86" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
+        <v>46239</v>
+      </c>
       <c r="C86" s="9">
         <f>_xlfn.XLOOKUP(Log!A86, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E86" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D86" s="9">
+        <v>0.48472222222222222</v>
+      </c>
+      <c r="E86" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H86" s="2" t="str">
+        <v>1.9999999999999929</v>
+      </c>
+      <c r="F86" s="7">
+        <v>30</v>
+      </c>
+      <c r="G86" s="2">
+        <v>31</v>
+      </c>
+      <c r="H86" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="87" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
+        <v>46239</v>
+      </c>
       <c r="C87" s="9">
         <f>_xlfn.XLOOKUP(Log!A87, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E87" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D87" s="9">
+        <v>0.48716435185185186</v>
+      </c>
+      <c r="E87" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H87" s="2" t="str">
+        <v>5.5166666666666764</v>
+      </c>
+      <c r="F87" s="7">
+        <v>38</v>
+      </c>
+      <c r="G87" s="2">
+        <v>39</v>
+      </c>
+      <c r="H87" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="88" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
+        <v>46239</v>
+      </c>
       <c r="C88" s="9">
         <f>_xlfn.XLOOKUP(Log!A88, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E88" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D88" s="9">
+        <v>0.48856481481481484</v>
+      </c>
+      <c r="E88" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H88" s="2" t="str">
+        <v>7.5333333333333652</v>
+      </c>
+      <c r="F88" s="7">
+        <v>41</v>
+      </c>
+      <c r="G88" s="2">
+        <v>42</v>
+      </c>
+      <c r="H88" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="89" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
+        <v>46239</v>
+      </c>
       <c r="C89" s="9">
         <f>_xlfn.XLOOKUP(Log!A89, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E89" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D89" s="9">
+        <v>0.48995370370370372</v>
+      </c>
+      <c r="E89" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H89" s="2" t="str">
+        <v>9.5333333333333581</v>
+      </c>
+      <c r="F89" s="7">
+        <v>42</v>
+      </c>
+      <c r="G89" s="2">
+        <v>45</v>
+      </c>
+      <c r="H89" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="90" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A90" s="1">
+        <v>46239</v>
+      </c>
       <c r="C90" s="9">
         <f>_xlfn.XLOOKUP(Log!A90, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E90" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D90" s="9">
+        <v>0.49135416666666665</v>
+      </c>
+      <c r="E90" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H90" s="2" t="str">
+        <v>11.549999999999967</v>
+      </c>
+      <c r="F90" s="7">
+        <v>44</v>
+      </c>
+      <c r="G90" s="2">
+        <v>47</v>
+      </c>
+      <c r="H90" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A91" s="1">
+        <v>46239</v>
+      </c>
       <c r="C91" s="9">
         <f>_xlfn.XLOOKUP(Log!A91, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E91" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D91" s="9">
+        <v>0.49275462962962963</v>
+      </c>
+      <c r="E91" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H91" s="2" t="str">
+        <v>13.566666666666656</v>
+      </c>
+      <c r="F91" s="7">
+        <v>47</v>
+      </c>
+      <c r="G91" s="2">
+        <v>48</v>
+      </c>
+      <c r="H91" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A92" s="1">
+        <v>46239</v>
+      </c>
       <c r="C92" s="9">
         <f>_xlfn.XLOOKUP(Log!A92, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E92" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D92" s="9">
+        <v>0.4941550925925926</v>
+      </c>
+      <c r="E92" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H92" s="2" t="str">
+        <v>15.583333333333345</v>
+      </c>
+      <c r="F92" s="7">
+        <v>48</v>
+      </c>
+      <c r="G92" s="2">
+        <v>49</v>
+      </c>
+      <c r="H92" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A93" s="1">
+        <v>46239</v>
+      </c>
       <c r="C93" s="9">
         <f>_xlfn.XLOOKUP(Log!A93, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E93" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D93" s="9">
+        <v>0.49554398148148149</v>
+      </c>
+      <c r="E93" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H93" s="2" t="str">
+        <v>17.583333333333336</v>
+      </c>
+      <c r="F93" s="7">
+        <v>49</v>
+      </c>
+      <c r="G93" s="2">
+        <v>51</v>
+      </c>
+      <c r="H93" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="3:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A94" s="1">
+        <v>46239</v>
+      </c>
       <c r="C94" s="9">
         <f>_xlfn.XLOOKUP(Log!A94, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E94" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D94" s="9">
+        <v>0.49694444444444447</v>
+      </c>
+      <c r="E94" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H94" s="2" t="str">
+        <v>19.600000000000026</v>
+      </c>
+      <c r="F94" s="7">
+        <v>51</v>
+      </c>
+      <c r="G94" s="2">
+        <v>52</v>
+      </c>
+      <c r="H94" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="95" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A95" s="1">
+        <v>46239</v>
+      </c>
       <c r="C95" s="9">
         <f>_xlfn.XLOOKUP(Log!A95, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E95" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D95" s="9">
+        <v>0.49833333333333335</v>
+      </c>
+      <c r="E95" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H95" s="2" t="str">
+        <v>21.600000000000019</v>
+      </c>
+      <c r="F95" s="7">
+        <v>51</v>
+      </c>
+      <c r="G95" s="2">
+        <v>54</v>
+      </c>
+      <c r="H95" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="96" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A96" s="1">
+        <v>46239</v>
+      </c>
       <c r="C96" s="9">
         <f>_xlfn.XLOOKUP(Log!A96, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E96" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D96" s="9">
+        <v>0.49972222222222223</v>
+      </c>
+      <c r="E96" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H96" s="2" t="str">
+        <v>23.600000000000012</v>
+      </c>
+      <c r="F96" s="7">
+        <v>52</v>
+      </c>
+      <c r="G96" s="2">
+        <v>55</v>
+      </c>
+      <c r="H96" s="2">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="97" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A97" s="1">
+        <v>46239</v>
+      </c>
       <c r="C97" s="9">
         <f>_xlfn.XLOOKUP(Log!A97, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E97" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D97" s="9">
+        <v>0.50111111111111106</v>
+      </c>
+      <c r="E97" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H97" s="2" t="str">
+        <v>25.599999999999923</v>
+      </c>
+      <c r="F97" s="7">
+        <v>54</v>
+      </c>
+      <c r="G97" s="2">
+        <v>55</v>
+      </c>
+      <c r="H97" s="2">
         <f t="shared" ref="H97:H160" si="5">IF(AND(G97&lt;&gt;"",F97&lt;&gt;""),G97-F97,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A98" s="1">
+        <v>46239</v>
+      </c>
       <c r="C98" s="9">
         <f>_xlfn.XLOOKUP(Log!A98, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E98" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D98" s="9">
+        <v>0.5025115740740741</v>
+      </c>
+      <c r="E98" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H98" s="2" t="str">
+        <v>27.616666666666696</v>
+      </c>
+      <c r="F98" s="7">
+        <v>54</v>
+      </c>
+      <c r="G98" s="2">
+        <v>57</v>
+      </c>
+      <c r="H98" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="99" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A99" s="1">
+        <v>46239</v>
+      </c>
       <c r="C99" s="9">
         <f>_xlfn.XLOOKUP(Log!A99, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E99" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D99" s="9">
+        <v>0.50391203703703702</v>
+      </c>
+      <c r="E99" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H99" s="2" t="str">
+        <v>29.633333333333304</v>
+      </c>
+      <c r="F99" s="7">
+        <v>55</v>
+      </c>
+      <c r="G99" s="2">
+        <v>57</v>
+      </c>
+      <c r="H99" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="100" spans="3:8" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A100" s="1">
+        <v>46239</v>
+      </c>
       <c r="C100" s="9">
         <f>_xlfn.XLOOKUP(Log!A100, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E100" s="6" t="str">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="D100" s="9">
+        <v>0.5053009259259259</v>
+      </c>
+      <c r="E100" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H100" s="2" t="str">
+        <v>31.633333333333297</v>
+      </c>
+      <c r="F100" s="7">
+        <v>55</v>
+      </c>
+      <c r="G100" s="2">
+        <v>58</v>
+      </c>
+      <c r="H100" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="101" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C101" s="9">
         <f>_xlfn.XLOOKUP(Log!A101, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -5999,7 +6285,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C102" s="9">
         <f>_xlfn.XLOOKUP(Log!A102, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6013,7 +6299,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C103" s="9">
         <f>_xlfn.XLOOKUP(Log!A103, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6027,7 +6313,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C104" s="9">
         <f>_xlfn.XLOOKUP(Log!A104, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6041,7 +6327,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C105" s="9">
         <f>_xlfn.XLOOKUP(Log!A105, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6055,7 +6341,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C106" s="9">
         <f>_xlfn.XLOOKUP(Log!A106, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6069,7 +6355,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C107" s="9">
         <f>_xlfn.XLOOKUP(Log!A107, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6083,7 +6369,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C108" s="9">
         <f>_xlfn.XLOOKUP(Log!A108, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6097,7 +6383,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C109" s="9">
         <f>_xlfn.XLOOKUP(Log!A109, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6111,7 +6397,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C110" s="9">
         <f>_xlfn.XLOOKUP(Log!A110, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6125,7 +6411,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C111" s="9">
         <f>_xlfn.XLOOKUP(Log!A111, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6139,7 +6425,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C112" s="9">
         <f>_xlfn.XLOOKUP(Log!A112, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -12160,7 +12446,7 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="D3:XFD32 D33:L40 D41:XFD44 D45:H45 D46:XFD1048576 A1 I1:XFD1 D2:I2 K2:XFD2 O33:XFD40 J45:XFD45 A2:C1048576">
+  <conditionalFormatting sqref="A2:C1048576 D3:XFD32 D33:L40 D41:XFD44 D45:H45 D46:XFD1048576 A1 I1:XFD1 D2:I2 K2:XFD2 O33:XFD40 J45:XFD45">
     <cfRule type="expression" dxfId="2" priority="2">
       <formula>AND(ROW()&gt;2, COLUMN()&lt;8, MOD(ROW(),2)=0)</formula>
     </cfRule>
@@ -12386,7 +12672,7 @@
         <f>IF(AND(D10&lt;&gt;"", C10&lt;&gt;""), IF(COUNTIFS(Log!$A$3:$A$9999,B10,Log!$F$3:$F$9999,"&gt;=50")=0,"–",_xlfn.MINIFS(Log!$E$3:$E$9999,Log!$A$3:$A$9999,B10,Log!$F$3:$F$9999,"&gt;=50")), "")</f>
         <v>21.583333333333243</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="27" t="s">
         <v>44</v>
       </c>
     </row>
@@ -12408,7 +12694,7 @@
         <v>21.216666666666654</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>46238</v>
       </c>
@@ -12421,20 +12707,33 @@
       <c r="D12" s="8">
         <v>0.42986111111111114</v>
       </c>
-      <c r="E12" s="25" t="str">
+      <c r="E12" s="25">
         <f>IF(AND(D12&lt;&gt;"", C12&lt;&gt;""), IF(COUNTIFS(Log!$A$3:$A$9999,B12,Log!$F$3:$F$9999,"&gt;=50")=0,"–",_xlfn.MINIFS(Log!$E$3:$E$9999,Log!$A$3:$A$9999,B12,Log!$F$3:$F$9999,"&gt;=50")), "")</f>
-        <v>–</v>
+        <v>21.066666666666627</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="E13" s="25" t="str">
+      <c r="A13" s="1">
+        <v>46239</v>
+      </c>
+      <c r="B13" s="1">
+        <v>46239</v>
+      </c>
+      <c r="C13" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="D13" s="8">
+        <v>0.48333333333333334</v>
+      </c>
+      <c r="E13" s="25">
         <f>IF(AND(D13&lt;&gt;"", C13&lt;&gt;""), IF(COUNTIFS(Log!$A$3:$A$9999,B13,Log!$F$3:$F$9999,"&gt;=50")=0,"–",_xlfn.MINIFS(Log!$E$3:$E$9999,Log!$A$3:$A$9999,B13,Log!$F$3:$F$9999,"&gt;=50")), "")</f>
-        <v/>
+        <v>19.600000000000026</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -13108,185 +13407,191 @@
   <dimension ref="A1:Y7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.77734375" style="43" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" style="41"/>
-    <col min="3" max="20" width="6.77734375" style="42" customWidth="1"/>
-    <col min="21" max="21" width="2.77734375" style="38" customWidth="1"/>
-    <col min="22" max="22" width="8.88671875" style="39"/>
-    <col min="23" max="25" width="10.77734375" style="38" customWidth="1"/>
-    <col min="26" max="16384" width="8.88671875" style="38"/>
+    <col min="1" max="1" width="25.77734375" style="41" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="39"/>
+    <col min="3" max="20" width="6.77734375" style="40" customWidth="1"/>
+    <col min="21" max="21" width="2.77734375" style="36" customWidth="1"/>
+    <col min="22" max="22" width="8.88671875" style="37"/>
+    <col min="23" max="25" width="10.77734375" style="36" customWidth="1"/>
+    <col min="26" max="16384" width="8.88671875" style="36"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="31" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:25" s="30" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="V1" s="31"/>
+    </row>
+    <row r="2" spans="1:25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="V1" s="32"/>
-    </row>
-    <row r="2" spans="1:25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="49"/>
+      <c r="R2" s="49"/>
+      <c r="S2" s="49"/>
+      <c r="T2" s="50"/>
+      <c r="V2" s="32"/>
+    </row>
+    <row r="3" spans="1:25" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="35" t="str" cm="1">
+        <f t="array" ref="C3:T3">LEFT(TRANSPOSE('[1]Data-Lists'!A2:A19), 3)</f>
+        <v xml:space="preserve">#1 </v>
+      </c>
+      <c r="D3" s="35" t="str">
+        <v xml:space="preserve">#2 </v>
+      </c>
+      <c r="E3" s="35" t="str">
+        <v xml:space="preserve">#3 </v>
+      </c>
+      <c r="F3" s="35" t="str">
+        <v xml:space="preserve">#4 </v>
+      </c>
+      <c r="G3" s="35" t="str">
+        <v xml:space="preserve">#5 </v>
+      </c>
+      <c r="H3" s="35" t="str">
+        <v xml:space="preserve">#6 </v>
+      </c>
+      <c r="I3" s="46" t="str">
+        <v xml:space="preserve">#7 </v>
+      </c>
+      <c r="J3" s="46" t="str">
+        <v xml:space="preserve">#8 </v>
+      </c>
+      <c r="K3" s="35" t="str">
+        <v xml:space="preserve">#9 </v>
+      </c>
+      <c r="L3" s="35" t="str">
+        <v>#10</v>
+      </c>
+      <c r="M3" s="35" t="str">
+        <v>#11</v>
+      </c>
+      <c r="N3" s="35" t="str">
+        <v>#12</v>
+      </c>
+      <c r="O3" s="46" t="str">
+        <v>#13</v>
+      </c>
+      <c r="P3" s="35" t="str">
+        <v>#14</v>
+      </c>
+      <c r="Q3" s="35" t="str">
+        <v>#15</v>
+      </c>
+      <c r="R3" s="35" t="str">
+        <v>#16</v>
+      </c>
+      <c r="S3" s="35" t="str">
+        <v>#17</v>
+      </c>
+      <c r="T3" s="35" t="str">
+        <v>#18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A4" s="38">
+        <v>46238</v>
+      </c>
+      <c r="C4" s="42">
+        <v>5</v>
+      </c>
+      <c r="D4" s="42">
+        <v>5</v>
+      </c>
+      <c r="E4" s="42">
+        <v>2</v>
+      </c>
+      <c r="F4" s="42">
+        <v>2</v>
+      </c>
+      <c r="G4" s="42">
+        <v>2</v>
+      </c>
+      <c r="H4" s="42">
+        <v>2</v>
+      </c>
+      <c r="I4" s="42">
+        <v>2</v>
+      </c>
+      <c r="J4" s="42">
+        <v>2</v>
+      </c>
+      <c r="K4" s="42">
+        <v>2</v>
+      </c>
+      <c r="L4" s="42"/>
+      <c r="M4" s="42"/>
+      <c r="N4" s="42"/>
+      <c r="O4" s="42"/>
+      <c r="P4" s="42"/>
+      <c r="Q4" s="42"/>
+      <c r="R4" s="42">
+        <v>1</v>
+      </c>
+      <c r="S4" s="42">
+        <v>1</v>
+      </c>
+      <c r="T4" s="42">
+        <v>2</v>
+      </c>
+      <c r="W4" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
-      <c r="R2" s="46"/>
-      <c r="S2" s="46"/>
-      <c r="T2" s="47"/>
-      <c r="V2" s="33"/>
-    </row>
-    <row r="3" spans="1:25" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="36" t="str" cm="1">
-        <f t="array" ref="C3:T3">LEFT(TRANSPOSE([1]Lists!A2:A19), 3)</f>
-        <v xml:space="preserve">#1 </v>
-      </c>
-      <c r="D3" s="36" t="str">
-        <v xml:space="preserve">#2 </v>
-      </c>
-      <c r="E3" s="36" t="str">
-        <v xml:space="preserve">#3 </v>
-      </c>
-      <c r="F3" s="36" t="str">
-        <v xml:space="preserve">#4 </v>
-      </c>
-      <c r="G3" s="36" t="str">
-        <v xml:space="preserve">#5 </v>
-      </c>
-      <c r="H3" s="36" t="str">
-        <v xml:space="preserve">#6 </v>
-      </c>
-      <c r="I3" s="36" t="str">
-        <v xml:space="preserve">#7 </v>
-      </c>
-      <c r="J3" s="37" t="str">
-        <v xml:space="preserve">#8 </v>
-      </c>
-      <c r="K3" s="36" t="str">
-        <v xml:space="preserve">#9 </v>
-      </c>
-      <c r="L3" s="36" t="str">
-        <v>#10</v>
-      </c>
-      <c r="M3" s="36" t="str">
-        <v>#11</v>
-      </c>
-      <c r="N3" s="36" t="str">
-        <v>#12</v>
-      </c>
-      <c r="O3" s="37" t="str">
-        <v>#13</v>
-      </c>
-      <c r="P3" s="36" t="str">
-        <v>#14</v>
-      </c>
-      <c r="Q3" s="36" t="str">
-        <v>#15</v>
-      </c>
-      <c r="R3" s="36" t="str">
-        <v>#16</v>
-      </c>
-      <c r="S3" s="36" t="str">
-        <v>#17</v>
-      </c>
-      <c r="T3" s="36" t="str">
-        <v>#18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A4" s="40">
-        <v>46238</v>
-      </c>
-      <c r="C4" s="44">
-        <v>3</v>
-      </c>
-      <c r="D4" s="44">
-        <v>3</v>
-      </c>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="44"/>
-      <c r="M4" s="44"/>
-      <c r="N4" s="44"/>
-      <c r="O4" s="44"/>
-      <c r="P4" s="44"/>
-      <c r="Q4" s="44"/>
-      <c r="R4" s="44">
-        <v>1</v>
-      </c>
-      <c r="S4" s="44">
-        <v>1</v>
-      </c>
-      <c r="T4" s="44">
-        <v>2</v>
-      </c>
-      <c r="V4" s="48"/>
-      <c r="W4" s="52" t="s">
-        <v>50</v>
-      </c>
-      <c r="X4" s="51"/>
-      <c r="Y4" s="51"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="44"/>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A5" s="40"/>
-      <c r="V5" s="48"/>
-      <c r="W5" s="50"/>
-      <c r="X5" s="50"/>
-      <c r="Y5" s="49"/>
+      <c r="A5" s="38"/>
+      <c r="W5" s="43"/>
+      <c r="X5" s="43"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="V6" s="48"/>
-      <c r="W6" s="49"/>
-      <c r="X6" s="50"/>
-      <c r="Y6" s="49"/>
+      <c r="X6" s="43"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="V7" s="48"/>
-      <c r="W7" s="50"/>
-      <c r="X7" s="50"/>
-      <c r="Y7" s="49"/>
+      <c r="W7" s="43"/>
+      <c r="X7" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
08/08/26 16:27 sync update
</commit_message>
<xml_diff>
--- a/Documentation Data/LCAS Vicon Temperature Tracker.xlsx
+++ b/Documentation Data/LCAS Vicon Temperature Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newwb\Documents\brain\professional\university\LCAS\EPSURIS Internship (Vicon)\Public Files\Documentation Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9030D01B-764E-4BC0-A0CE-D8E29AA06B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683BE9AF-6F55-491E-9784-81250A6FE53E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="4" r:id="rId1"/>
@@ -1260,6 +1260,9 @@
                 <c:pt idx="10">
                   <c:v>46239</c:v>
                 </c:pt>
+                <c:pt idx="11">
+                  <c:v>46240</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1301,6 +1304,9 @@
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>24.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>24</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1387,6 +1393,9 @@
                 <c:pt idx="10">
                   <c:v>46239</c:v>
                 </c:pt>
+                <c:pt idx="11">
+                  <c:v>46240</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1430,7 +1439,7 @@
                   <c:v>19.600000000000026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>20.133333333333336</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
@@ -3174,17 +3183,18 @@
       <xxl21:absoluteUrl r:id="rId2"/>
     </xxl21:alternateUrls>
     <sheetNames>
-      <sheetName val="Instructions"/>
+      <sheetName val="WIP"/>
       <sheetName val="Data-Lists"/>
-      <sheetName val="Camera Labelling"/>
-      <sheetName val="Log"/>
-      <sheetName val="Daily Summary"/>
+      <sheetName val="Labelling"/>
+      <sheetName val="Daily Log"/>
+      <sheetName val="Secondary Log"/>
+      <sheetName val="Daily Recap"/>
+      <sheetName val="Trial Recap"/>
+      <sheetName val="Error Recap"/>
       <sheetName val="Camera Error Trend"/>
       <sheetName val="Camera Performance Trends"/>
       <sheetName val="High Error Cameras"/>
       <sheetName val="Problem Cameras"/>
-      <sheetName val="Error Log"/>
-      <sheetName val="Error Summary"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -3289,6 +3299,7 @@
       <sheetData sheetId="8"/>
       <sheetData sheetId="9"/>
       <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -6272,230 +6283,422 @@
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A101" s="1">
+        <v>46240</v>
+      </c>
       <c r="C101" s="9">
         <f>_xlfn.XLOOKUP(Log!A101, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E101" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D101" s="9">
+        <v>0.44027777777777777</v>
+      </c>
+      <c r="E101" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H101" s="2" t="str">
+        <v>1.9999999999999929</v>
+      </c>
+      <c r="F101" s="7">
+        <v>32</v>
+      </c>
+      <c r="G101" s="2">
+        <v>33</v>
+      </c>
+      <c r="H101" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A102" s="1">
+        <v>46240</v>
+      </c>
       <c r="C102" s="9">
         <f>_xlfn.XLOOKUP(Log!A102, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E102" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D102" s="9">
+        <v>0.44170138888888888</v>
+      </c>
+      <c r="E102" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H102" s="2" t="str">
+        <v>4.0499999999999936</v>
+      </c>
+      <c r="F102" s="7">
+        <v>35</v>
+      </c>
+      <c r="G102" s="2">
+        <v>36</v>
+      </c>
+      <c r="H102" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
+        <v>46240</v>
+      </c>
       <c r="C103" s="9">
         <f>_xlfn.XLOOKUP(Log!A103, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E103" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D103" s="9">
+        <v>0.44310185185185186</v>
+      </c>
+      <c r="E103" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H103" s="2" t="str">
+        <v>6.0666666666666824</v>
+      </c>
+      <c r="F103" s="7">
+        <v>38</v>
+      </c>
+      <c r="G103" s="2">
+        <v>41</v>
+      </c>
+      <c r="H103" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A104" s="1">
+        <v>46240</v>
+      </c>
       <c r="C104" s="9">
         <f>_xlfn.XLOOKUP(Log!A104, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E104" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D104" s="9">
+        <v>0.44450231481481484</v>
+      </c>
+      <c r="E104" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H104" s="2" t="str">
+        <v>8.0833333333333712</v>
+      </c>
+      <c r="F104" s="7">
+        <v>41</v>
+      </c>
+      <c r="G104" s="2">
+        <v>44</v>
+      </c>
+      <c r="H104" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A105" s="1">
+        <v>46240</v>
+      </c>
       <c r="C105" s="9">
         <f>_xlfn.XLOOKUP(Log!A105, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E105" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D105" s="9">
+        <v>0.44590277777777776</v>
+      </c>
+      <c r="E105" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H105" s="2" t="str">
+        <v>10.09999999999998</v>
+      </c>
+      <c r="F105" s="7">
+        <v>44</v>
+      </c>
+      <c r="G105" s="2">
+        <v>45</v>
+      </c>
+      <c r="H105" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A106" s="1">
+        <v>46240</v>
+      </c>
       <c r="C106" s="9">
         <f>_xlfn.XLOOKUP(Log!A106, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E106" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D106" s="9">
+        <v>0.44729166666666664</v>
+      </c>
+      <c r="E106" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H106" s="2" t="str">
+        <v>12.099999999999973</v>
+      </c>
+      <c r="F106" s="7">
+        <v>44</v>
+      </c>
+      <c r="G106" s="2">
+        <v>47</v>
+      </c>
+      <c r="H106" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A107" s="1">
+        <v>46240</v>
+      </c>
       <c r="C107" s="9">
         <f>_xlfn.XLOOKUP(Log!A107, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E107" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D107" s="9">
+        <v>0.44868055555555558</v>
+      </c>
+      <c r="E107" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H107" s="2" t="str">
+        <v>14.100000000000046</v>
+      </c>
+      <c r="F107" s="7">
+        <v>47</v>
+      </c>
+      <c r="G107" s="2">
+        <v>49</v>
+      </c>
+      <c r="H107" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A108" s="1">
+        <v>46240</v>
+      </c>
       <c r="C108" s="9">
         <f>_xlfn.XLOOKUP(Log!A108, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E108" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D108" s="9">
+        <v>0.45008101851851851</v>
+      </c>
+      <c r="E108" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H108" s="2" t="str">
+        <v>16.116666666666653</v>
+      </c>
+      <c r="F108" s="7">
+        <v>48</v>
+      </c>
+      <c r="G108" s="2">
+        <v>51</v>
+      </c>
+      <c r="H108" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A109" s="1">
+        <v>46240</v>
+      </c>
       <c r="C109" s="9">
         <f>_xlfn.XLOOKUP(Log!A109, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E109" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D109" s="9">
+        <v>0.45148148148148148</v>
+      </c>
+      <c r="E109" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H109" s="2" t="str">
+        <v>18.133333333333344</v>
+      </c>
+      <c r="F109" s="7">
+        <v>49</v>
+      </c>
+      <c r="G109" s="2">
+        <v>52</v>
+      </c>
+      <c r="H109" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A110" s="1">
+        <v>46240</v>
+      </c>
       <c r="C110" s="9">
         <f>_xlfn.XLOOKUP(Log!A110, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E110" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D110" s="9">
+        <v>0.45287037037037037</v>
+      </c>
+      <c r="E110" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H110" s="2" t="str">
+        <v>20.133333333333336</v>
+      </c>
+      <c r="F110" s="7">
+        <v>51</v>
+      </c>
+      <c r="G110" s="2">
+        <v>52</v>
+      </c>
+      <c r="H110" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A111" s="1">
+        <v>46240</v>
+      </c>
       <c r="C111" s="9">
         <f>_xlfn.XLOOKUP(Log!A111, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E111" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D111" s="9">
+        <v>0.45425925925925925</v>
+      </c>
+      <c r="E111" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H111" s="2" t="str">
+        <v>22.133333333333329</v>
+      </c>
+      <c r="F111" s="7">
+        <v>51</v>
+      </c>
+      <c r="G111" s="2">
+        <v>54</v>
+      </c>
+      <c r="H111" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A112" s="1">
+        <v>46240</v>
+      </c>
       <c r="C112" s="9">
         <f>_xlfn.XLOOKUP(Log!A112, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E112" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D112" s="9">
+        <v>0.45565972222222223</v>
+      </c>
+      <c r="E112" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H112" s="2" t="str">
+        <v>24.15000000000002</v>
+      </c>
+      <c r="F112" s="7">
+        <v>52</v>
+      </c>
+      <c r="G112" s="2">
+        <v>55</v>
+      </c>
+      <c r="H112" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="113" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A113" s="1">
+        <v>46240</v>
+      </c>
       <c r="C113" s="9">
         <f>_xlfn.XLOOKUP(Log!A113, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E113" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D113" s="9">
+        <v>0.45704861111111111</v>
+      </c>
+      <c r="E113" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H113" s="2" t="str">
+        <v>26.150000000000013</v>
+      </c>
+      <c r="F113" s="7">
+        <v>54</v>
+      </c>
+      <c r="G113" s="2">
+        <v>55</v>
+      </c>
+      <c r="H113" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="114" spans="3:8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A114" s="1">
+        <v>46240</v>
+      </c>
       <c r="C114" s="9">
         <f>_xlfn.XLOOKUP(Log!A114, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E114" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D114" s="9">
+        <v>0.4584375</v>
+      </c>
+      <c r="E114" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H114" s="2" t="str">
+        <v>28.150000000000006</v>
+      </c>
+      <c r="F114" s="7">
+        <v>54</v>
+      </c>
+      <c r="G114" s="2">
+        <v>57</v>
+      </c>
+      <c r="H114" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="115" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A115" s="1">
+        <v>46240</v>
+      </c>
       <c r="C115" s="9">
         <f>_xlfn.XLOOKUP(Log!A115, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E115" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D115" s="9">
+        <v>0.45983796296296298</v>
+      </c>
+      <c r="E115" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H115" s="2" t="str">
+        <v>30.166666666666693</v>
+      </c>
+      <c r="F115" s="7">
+        <v>55</v>
+      </c>
+      <c r="G115" s="2">
+        <v>58</v>
+      </c>
+      <c r="H115" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="116" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A116" s="1">
+        <v>46240</v>
+      </c>
       <c r="C116" s="9">
         <f>_xlfn.XLOOKUP(Log!A116, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
-        <v>0</v>
-      </c>
-      <c r="E116" s="6" t="str">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="D116" s="9">
+        <v>0.46122685185185186</v>
+      </c>
+      <c r="E116" s="6">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H116" s="2" t="str">
+        <v>32.166666666666686</v>
+      </c>
+      <c r="F116" s="7">
+        <v>55</v>
+      </c>
+      <c r="G116" s="2">
+        <v>58</v>
+      </c>
+      <c r="H116" s="2">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="117" spans="3:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C117" s="9">
         <f>_xlfn.XLOOKUP(Log!A117, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6509,7 +6712,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C118" s="9">
         <f>_xlfn.XLOOKUP(Log!A118, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6523,7 +6726,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C119" s="9">
         <f>_xlfn.XLOOKUP(Log!A119, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6537,7 +6740,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C120" s="9">
         <f>_xlfn.XLOOKUP(Log!A120, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6551,7 +6754,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C121" s="9">
         <f>_xlfn.XLOOKUP(Log!A121, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6565,7 +6768,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C122" s="9">
         <f>_xlfn.XLOOKUP(Log!A122, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6579,7 +6782,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C123" s="9">
         <f>_xlfn.XLOOKUP(Log!A123, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6593,7 +6796,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C124" s="9">
         <f>_xlfn.XLOOKUP(Log!A124, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6607,7 +6810,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C125" s="9">
         <f>_xlfn.XLOOKUP(Log!A125, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6621,7 +6824,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C126" s="9">
         <f>_xlfn.XLOOKUP(Log!A126, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6635,7 +6838,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C127" s="9">
         <f>_xlfn.XLOOKUP(Log!A127, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -6649,7 +6852,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C128" s="9">
         <f>_xlfn.XLOOKUP(Log!A128, 'Daily Summary'!A:A, 'Daily Summary'!D:D, "Not found!")</f>
         <v>0</v>
@@ -12446,7 +12649,7 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="A2:C1048576 D3:XFD32 D33:L40 D41:XFD44 D45:H45 D46:XFD1048576 A1 I1:XFD1 D2:I2 K2:XFD2 O33:XFD40 J45:XFD45">
+  <conditionalFormatting sqref="D3:XFD32 D33:L40 D41:XFD44 D45:H45 D46:XFD1048576 A1 I1:XFD1 D2:I2 K2:XFD2 O33:XFD40 J45:XFD45 A2:C1048576">
     <cfRule type="expression" dxfId="2" priority="2">
       <formula>AND(ROW()&gt;2, COLUMN()&lt;8, MOD(ROW(),2)=0)</formula>
     </cfRule>
@@ -12737,11 +12940,21 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="E14" s="25" t="str">
+      <c r="A14" s="1">
+        <v>46240</v>
+      </c>
+      <c r="B14" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C14" s="2">
+        <v>24</v>
+      </c>
+      <c r="D14" s="8">
+        <v>0.43888888888888888</v>
+      </c>
+      <c r="E14" s="25">
         <f>IF(AND(D14&lt;&gt;"", C14&lt;&gt;""), IF(COUNTIFS(Log!$A$3:$A$9999,B14,Log!$F$3:$F$9999,"&gt;=50")=0,"–",_xlfn.MINIFS(Log!$E$3:$E$9999,Log!$A$3:$A$9999,B14,Log!$F$3:$F$9999,"&gt;=50")), "")</f>
-        <v/>
+        <v>20.133333333333336</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>